<commit_message>
HU-028: correcciones en la guia LWC+Apex y memoria del proyecto
Guia (planilla): fila de PA corregida (listas administradas en SAP, PBE solo
referencia, precedencia pendiente con Grupo Q); nueva fila de Combos (SKU
propio con precio del SAP, sin CPQ); seccion 'Guardas de licenciamiento y
fronteras' en Estandares (sin CPQ/Revenue Cloud/EPC; carga masiva en SAP;
simulador y comparacion exigen servicio en el contrato MuleSoft).

CLAUDE.md: proceso de validacion de HUs antes del refinamiento (compromiso
con Melisa) y guardas de licenciamiento/arquitectura para no repetir en
ninguna HU.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -878,12 +878,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compatibilidad por modelo/marca &gt; precio (PricebookEntry o SAP) &gt; Order &gt; SAP</t>
+          <t xml:space="preserve">Compatibilidad por modelo/marca &gt; precio: SAP resuelve la lista aplicable (general/canal/cliente/volumen, con vigencia) &gt; Order &gt; SAP</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PA puede ir por PricebookEntry (no siempre real-time)</t>
+          <t xml:space="preserve">Listas de PA administradas en SAP (HU-028); PBE solo referencia de exhibicion. Precedencia de listas: pendiente confirmar con Grupo Q</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -895,25 +895,52 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Combos (SKU con precio propio)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dentro de Repuestos/PA</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El combo es un Product2 propio (ProductCode=material SAP); SAP resuelve su precio como cualquier material; disponibilidad del kit en HU-043</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO requiere CPQ; la composicion no afecta el precio</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Si aplica</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Nuevo flujo (escalable)</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Nuevo hijo LWC</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Reusa la capa de servicio Apex; solo cambia la UI</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Igual</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Igual</t>
         </is>
@@ -1183,12 +1210,57 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limite a tener presente</t>
+          <t xml:space="preserve">Guardas de licenciamiento y fronteras (no olvidar)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GrupoQ NO tiene CPQ, Revenue Cloud ni EPC. Ninguna HU debe asumirlos (HU-028 corregida: precio de combos y listas se resuelven en SAP + objetos estandar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra (no calcula ni convierte moneda). Listas de PA administradas en SAP; PBE solo referencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carga masiva de precios/parametros de pricing: es del SAP (los datos viven alla). No construir herramienta de carga en Salesforce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulador de precios (FOB/factor/mark-up): variables viven en SAP; si Grupo Q quiere UI en Salesforce, exige servicio de simulacion expuesto por MuleSoft (agregar al contrato de integracion).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comparacion de precios multi-canal/sociedad: el endpoint del Mule debe aceptar consulta multi-contexto (agregar al contrato de integracion).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limite a tener presente</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuation con Named Credential funciona con auth de sistema (client credentials / API key). Si el Mule exige OAuth por-usuario, ajustar la estrategia de auth antes.</t>
         </is>

</xml_diff>

<commit_message>
HU-039 validada: contrato MuleSoft y exclusion de Case en la guia; evidencia de licencias en memoria
Guia: dos guardas nuevas en Estandares — servicio de creacion/extension de
material (escritura de dato maestro en SAP, upsert Product2 por ProductCode)
y exclusion de Case en HUs de Repuestos (objeto custom + Record Types +
Queues + Duplicate Rules nativas).

CLAUDE.md: evidencia de licencias de la org (Salesforce Pricing 1+1 token vs
BRE 27.131 — no usar Price Management), exclusion de Case, y el servicio
nuevo de material en el contrato MuleSoft.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -1250,17 +1250,31 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23"/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Creacion/extension de material (HU-039): servicio nuevo en el contrato MuleSoft (verificar existencia por sociedad/centro + crear/extender). Es ESCRITURA de dato maestro en SAP: Salesforce solicita, SAP ejecuta y devuelve el codigo (MATNR) -&gt; upsert de Product2 por ProductCode.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Case esta EXCLUIDO de las HUs de Repuestos por decision del cliente (HU-039): solicitudes viven en objeto custom con Record Types + Queues + Duplicate Rules nativas + Files + Field History. Ninguna HU futura debe proponer Case sin validar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Limite a tener presente</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuation con Named Credential funciona con auth de sistema (client credentials / API key). Si el Mule exige OAuth por-usuario, ajustar la estrategia de auth antes.</t>
         </is>

</xml_diff>

<commit_message>
Guia de ventas: HU-039 reencuadrada como fuera del flujo de ventas
La creacion/extension de material pertenece al dominio de Gestion de
Productos (Annex fila 181), no al flujo de ventas. En la guia queda solo el
punto de contacto (busqueda sin resultado -> registrar solicitud -> la venta
continua); el servicio de dato maestro va al contrato MuleSoft del dominio
de productos.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -1252,29 +1252,22 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Creacion/extension de material (HU-039): servicio nuevo en el contrato MuleSoft (verificar existencia por sociedad/centro + crear/extender). Es ESCRITURA de dato maestro en SAP: Salesforce solicita, SAP ejecuta y devuelve el codigo (MATNR) -&gt; upsert de Product2 por ProductCode.</t>
+          <t xml:space="preserve">FUERA del flujo de ventas — dominio Gestion de Productos (HU-039): la creacion/extension de material NO es parte de este flujo. Unico punto de contacto: si la busqueda no encuentra el material, la UI ofrece registrar la solicitud y la venta continua. El servicio de escritura de dato maestro va al contrato MuleSoft del dominio de productos, no al de ventas.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Case esta EXCLUIDO de las HUs de Repuestos por decision del cliente (HU-039): solicitudes viven en objeto custom con Record Types + Queues + Duplicate Rules nativas + Files + Field History. Ninguna HU futura debe proponer Case sin validar.</t>
-        </is>
-      </c>
+      <c r="A24"/>
     </row>
     <row r="25">
-      <c r="A25"/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limite a tener presente</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Limite a tener presente</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuation con Named Credential funciona con auth de sistema (client credentials / API key). Si el Mule exige OAuth por-usuario, ajustar la estrategia de auth antes.</t>
         </is>

</xml_diff>

<commit_message>
Guia de ventas: comportamiento 'sin resultado' encajado en los flujos
Aba Flujos: nueva columna 'Si NO encuentra' por flujo — Venta Vehiculo usa
Vehicle Inventory Search en otras ubicaciones + Vehicle Transfer (unidad);
Contraventa/PA/B2B/Combos siguen el arbol de material (verificacion SAP,
upsert por ProductCode, extension automatica HU-039, solicitud prellenada o
Follow de la abierta; la venta sigue sin el item). Nueva fila Venta
Gestionada B2B (pipeline GQOpportunityProcessRepuestosPA). Aba Capas: nuevo
componente MaterialSearchService (comportamiento sin-resultado unico para
todos los flujos; la solicitud pertenece al dominio de productos).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -382,86 +382,108 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sap_Order_Response__e</t>
+          <t xml:space="preserve">MaterialSearchService</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platform Event</t>
+          <t xml:space="preserve">Apex</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Devuelve el resultado asincrono a la UI</t>
+          <t xml:space="preserve">Busqueda unificada: local (SOSL/Product2) &gt; verificacion SAP por sociedad/centro &gt; upsert por ProductCode &gt; extension automatica &gt; hand-off a solicitud (dominio Gestion de Productos)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">La LWC se suscribe con lightning/empApi</t>
+          <t xml:space="preserve">Un solo comportamiento sin-resultado para TODOS los flujos; la solicitud en si NO es del flujo de ventas</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow de assetizacion</t>
+          <t xml:space="preserve">Sap_Order_Response__e</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow record-triggered</t>
+          <t xml:space="preserve">Platform Event</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset + Vehicle (CurrentOwnerId) + Asset Contact Participant</t>
+          <t xml:space="preserve">Devuelve el resultado asincrono a la UI</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Declarativo, al activar el Order; sin objeto custom</t>
+          <t xml:space="preserve">La LWC se suscribe con lightning/empApi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ventaGuiadaAction</t>
+          <t xml:space="preserve">Flow de assetizacion</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LWC pai</t>
+          <t xml:space="preserve">Flow record-triggered</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Screen Quick Action; router por Record Type/contexto</t>
+          <t xml:space="preserve">Asset + Vehicle (CurrentOwnerId) + Asset Contact Participant</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">recordId por setter @api (no en connectedCallback)</t>
+          <t xml:space="preserve">Declarativo, al activar el Order; sin objeto custom</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">ventaGuiadaAction</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LWC pai</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Screen Quick Action; router por Record Type/contexto</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">recordId por setter @api (no en connectedCallback)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">ventaVehiculo / contraventaRepuestos / ventaPA</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">LWC hijos</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">UI especifica por flujo</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Finos; reusan la capa de servicio Apex</t>
         </is>
@@ -767,11 +789,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="52" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="32" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -810,6 +833,11 @@
           <t xml:space="preserve">Assetizacion</t>
         </is>
       </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Si NO encuentra (busqueda sin resultado)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -837,6 +865,11 @@
           <t xml:space="preserve">Asset + Vehicle + Asset Contact Participant (360)</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unidad no disponible en la sucursal: Vehicle Inventory Search en OTRAS ubicaciones + Vehicle Transfer (nativos, licenciados). Accesorios/PA dentro de la venta siguen el arbol de material</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -864,6 +897,11 @@
           <t xml:space="preserve">Solo unidades serializables/garantizables</t>
         </is>
       </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arbol de material: verifica SAP &gt; existe para sociedad/centro: upsert Product2 (ProductCode) y sigue &gt; existe sin centro: extension automatica (HU-039) &gt; no existe: solicitud prellenada o vincular a la abierta (Follow). La venta sigue sin ese item</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -891,64 +929,111 @@
           <t xml:space="preserve">Si es serializable</t>
         </is>
       </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mismo arbol de material que repuestos</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Combos (SKU con precio propio)</t>
+          <t xml:space="preserve">Venta Gestionada B2B (Repuestos &amp; PA)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dentro de Repuestos/PA</t>
+          <t xml:space="preserve">Opportunity pipeline GQOpportunityProcessRepuestosPA (mayoreo/flotas/cuentas clave/gobierno)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El combo es un Product2 propio (ProductCode=material SAP); SAP resuelve su precio como cualquier material; disponibilidad del kit en HU-043</t>
+          <t xml:space="preserve">Visita en campo &gt; cotizacion con vigencia &gt; negociacion &gt; Order &gt; SAP</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO requiere CPQ; la composicion no afecta el precio</t>
+          <t xml:space="preserve">Sync: consulta. Async: envio</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Si aplica</t>
+          <t xml:space="preserve">Si es serializable</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mismo arbol de material; ventaja: la solicitud se sigue (Follow) y el item se cotiza despues dentro de la vigencia de la cotizacion</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Combos (SKU con precio propio)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dentro de Repuestos/PA</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El combo es un Product2 propio (ProductCode=material SAP); SAP resuelve su precio como cualquier material; disponibilidad del kit en HU-043</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO requiere CPQ; la composicion no afecta el precio</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Si aplica</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combo no encontrado = mismo arbol de material (el combo es un material SAP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Nuevo flujo (escalable)</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Nuevo hijo LWC</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Reusa la capa de servicio Apex; solo cambia la UI</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Igual</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Igual</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reusa MaterialSearchService: el comportamiento sin-resultado es unico para todos los flujos</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Guia de ventas: flujo de Usados, colores de pestana y revision editorial completa
Nueva fila Venta de Usados en Flujos (inventario HU-045 propio o consignacion,
precio de la unidad administrado por Grupo Q, cotizacion y pedido a SAP,
nuevo Asset al comprador con ConditionType Antiguo; consignacion con Contract
RT Consignacion, comision y baja del inventario al cerrar). Hijo ventaUsados
en la capa de componentes y alerta de vencimiento del contrato en la hoja de
sincrono/asincrono. Las siete pestanas ahora llevan color; texto revisado en
espanol con acentuacion correcta. Cobertura completa de las cinco lineas de
negocio: Autos, Motos, Usados, Repuestos y PA.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Solucion" sheetId="1" r:id="rId1"/>
+    <sheet name="Solución" sheetId="1" r:id="rId1"/>
     <sheet name="Capas y componentes" sheetId="2" r:id="rId2"/>
     <sheet name="Paso a paso" sheetId="3" r:id="rId3"/>
     <sheet name="Flujos" sheetId="4" r:id="rId4"/>
-    <sheet name="Sync vs Async" sheetId="5" r:id="rId5"/>
-    <sheet name="Estandares" sheetId="6" r:id="rId6"/>
+    <sheet name="Síncrono vs Asíncrono" sheetId="5" r:id="rId5"/>
+    <sheet name="Estándares" sheetId="6" r:id="rId6"/>
     <sheet name="Referencias" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
@@ -124,14 +124,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF1F3864"/>
+  </sheetPr>
   <cols>
-    <col min="1" max="1" width="140" customWidth="1"/>
+    <col min="1" max="1" width="145" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arquitectura de Ventas — LWC + Apex (server-client) — Solucion firme</t>
+          <t xml:space="preserve">Arquitectura de Ventas — LWC + Apex (server-client)</t>
         </is>
       </c>
     </row>
@@ -141,7 +144,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solucion consolidada y alineada a los estandares de Salesforce. No cambia. LWC+Apex solo en UI e integracion; reglas de negocio en BRE; modelo, cotizacion, pedido y assetizacion en NATIVO. Consulta de precio+stock en tiempo real al SAP SIN bloqueo, via Apex Continuation.</t>
+          <t xml:space="preserve">Solución consolidada y alineada a los estándares de Salesforce. LWC y Apex se usan únicamente en la interfaz y en la capa de integración; las reglas de negocio viven en el motor de reglas (BRE); el modelo de datos, la cotización, el pedido y la assetización son nativos. La consulta de precio e inventario al SAP es en tiempo real y sin bloqueo, mediante Apex Continuation. Cubre las cinco líneas de negocio: Autos, Motos, Usados, Repuestos y PA.</t>
         </is>
       </c>
     </row>
@@ -151,56 +154,56 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Principios firmes</t>
+          <t xml:space="preserve">Principios</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Server-client: LWC (cliente, UX y orquestacion) + Apex (servidor).</t>
+          <t xml:space="preserve">1. Server-client: LWC en el cliente (experiencia y orquestación) y Apex en el servidor.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. Sincrono sin bloqueo: Apex Continuation (hasta 120s, hasta 3 callouts en paralelo, no bloquea la thread del app server). Es el mecanismo estandar para callout largo desde Lightning.</t>
+          <t xml:space="preserve">2. Síncrono sin bloqueo: Apex Continuation (hasta 120 segundos, hasta 3 callouts en paralelo, sin ocupar el hilo del servidor). Es el mecanismo estándar para callouts largos desde Lightning.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. Asincrono: Queueable + Platform Event + lightning/empApi (devuelve el resultado a la UI sin polling).</t>
+          <t xml:space="preserve">3. Asíncrono: Queueable + Platform Event + lightning/empApi, para devolver resultados a la interfaz sin polling.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. Reglas de precio/impuesto/exoneracion: BRE (Decision Matrix / Expression Set). Mantenido por el negocio, sin deploy. NO van a Apex.</t>
+          <t xml:space="preserve">4. Reglas de precio, impuesto y exoneración: Decision Matrix / Expression Set (BRE), mantenidas por el negocio sin despliegues. No se implementan en Apex.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5. Nativo: Quote &amp; Order Capture, Standalone Orders, Record Types, Asset / Vehicle / Asset Contact Participant. No se reescribe lo nativo.</t>
+          <t xml:space="preserve">5. Nativo: Quote and Order Capture, Standalone Orders, Record Types, Asset, Vehicle y Asset Contact Participant. Lo nativo no se reescribe.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6. Entrada: Screen Quick Action en la Oportunidad (venta de vehiculo) y Record Type dedicado para la contraventa de repuestos (balcon).</t>
+          <t xml:space="preserve">6. Puertas de entrada: acción de pantalla en la Oportunidad (vehículos nuevos y usados), Record Type dedicado para la contraventa de mostrador, y el mismo proceso transaccional expuesto como servicio para el canal online.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7. Cobertura: un componente pai (router) + hijos por flujo + una capa de servicio Apex compartida. Un flujo nuevo = un hijo nuevo, mismos servicios.</t>
+          <t xml:space="preserve">7. Cobertura: un componente padre (router) + un hijo por línea de negocio + una capa de servicios Apex compartida. Un flujo nuevo es un hijo nuevo; los servicios no se duplican.</t>
         </is>
       </c>
     </row>
@@ -217,30 +220,30 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apex/LWC: SOLO en UI e integracion.  |  BRE: reglas.  |  Nativo AC: catalogo, cotizacion, pedido, assetizacion.  |  SAP: autoridad fiscal y stock real.</t>
+          <t xml:space="preserve">LWC y Apex: solamente interfaz e integración.  |  BRE: reglas.  |  Nativo: catálogo, cotización, pedido y assetización.  |  SAP: autoridad fiscal, stock real y precio de Repuestos/PA.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:A1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF2E75B6"/>
+  </sheetPr>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capas y componentes (se construyen una vez, se reusan en todos los flujos)</t>
+          <t xml:space="preserve">Capas y componentes (se construyen una vez y los reutilizan todos los flujos)</t>
         </is>
       </c>
     </row>
@@ -265,7 +268,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nota tecnica</t>
+          <t xml:space="preserve">Nota técnica</t>
         </is>
       </c>
     </row>
@@ -277,17 +280,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Config</t>
+          <t xml:space="preserve">Configuración</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auth de sistema hacia MuleSoft/SAP</t>
+          <t xml:space="preserve">Autenticación de sistema hacia MuleSoft/SAP</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin credenciales en codigo; endpoint /api/v1/prices-and-inventory</t>
+          <t xml:space="preserve">Sin credenciales en el código; endpoint único de precios e inventario</t>
         </is>
       </c>
     </row>
@@ -304,12 +307,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consulta sincrona precio+stock al SAP</t>
+          <t xml:space="preserve">Consulta síncrona de precio y stock al SAP</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">@AuraEnabled(continuation=true cacheable=true) — espacio, no coma</t>
+          <t xml:space="preserve">@AuraEnabled(continuation=true cacheable=true) — con espacio, no coma</t>
         </is>
       </c>
     </row>
@@ -326,12 +329,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Invoca el BRE para precio/impuesto de referencia</t>
+          <t xml:space="preserve">Invoca el BRE para el precio e impuesto de referencia</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Las reglas viven en Decision Matrix/Expression Set, no en Apex</t>
+          <t xml:space="preserve">Las reglas viven en Decision Matrix / Expression Set, no en Apex</t>
         </is>
       </c>
     </row>
@@ -348,12 +351,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crea Quote/Order y line items por Record Type</t>
+          <t xml:space="preserve">Crea la cotización y el pedido según el Record Type</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DML bulkificado; nativo (Quote &amp; Order Capture / Standalone Orders)</t>
+          <t xml:space="preserve">DML bulkificado; Quote and Order Capture y Standalone Orders nativos</t>
         </is>
       </c>
     </row>
@@ -370,7 +373,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Envia el pedido al SAP (asincrono)</t>
+          <t xml:space="preserve">Envía el pedido al SAP de forma asíncrona</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -392,12 +395,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Busqueda unificada: local (SOSL/Product2) &gt; verificacion SAP por sociedad/centro &gt; upsert por ProductCode &gt; extension automatica &gt; hand-off a solicitud (dominio Gestion de Productos)</t>
+          <t xml:space="preserve">Búsqueda unificada: local (SOSL sobre Product2) &gt; verificación en SAP por sociedad/centro &gt; upsert por ProductCode &gt; extensión automática &gt; derivación a solicitud (dominio de Gestión de Productos)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Un solo comportamiento sin-resultado para TODOS los flujos; la solicitud en si NO es del flujo de ventas</t>
+          <t xml:space="preserve">Un solo comportamiento de 'sin resultado' para todos los flujos; la solicitud no pertenece al flujo de ventas</t>
         </is>
       </c>
     </row>
@@ -414,7 +417,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Devuelve el resultado asincrono a la UI</t>
+          <t xml:space="preserve">Devuelve el resultado asíncrono a la interfaz</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -426,7 +429,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow de assetizacion</t>
+          <t xml:space="preserve">Flow de assetización</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -441,7 +444,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Declarativo, al activar el Order; sin objeto custom</t>
+          <t xml:space="preserve">Declarativo, al activarse el pedido; sin objetos custom</t>
         </is>
       </c>
     </row>
@@ -453,24 +456,24 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LWC pai</t>
+          <t xml:space="preserve">LWC padre</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Screen Quick Action; router por Record Type/contexto</t>
+          <t xml:space="preserve">Acción de pantalla; enruta por Record Type y contexto</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">recordId por setter @api (no en connectedCallback)</t>
+          <t xml:space="preserve">recordId por setter @api (no llega en connectedCallback)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ventaVehiculo / contraventaRepuestos / ventaPA</t>
+          <t xml:space="preserve">ventaVehiculo / ventaUsados / contraventaRepuestos / ventaPA</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -480,35 +483,35 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">UI especifica por flujo</t>
+          <t xml:space="preserve">Interfaz específica de cada línea de negocio</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finos; reusan la capa de servicio Apex</t>
+          <t xml:space="preserve">Delgados; reutilizan la capa de servicios Apex</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF548235"/>
+  </sheetPr>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="3" max="3" width="62" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paso a paso de construccion (orden recomendado)</t>
+          <t xml:space="preserve">Paso a paso de construcción (orden recomendado)</t>
         </is>
       </c>
     </row>
@@ -528,12 +531,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Como</t>
+          <t xml:space="preserve">Cómo</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patron / Referencia</t>
+          <t xml:space="preserve">Patrón / referencia</t>
         </is>
       </c>
     </row>
@@ -545,12 +548,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Named Credential a MuleSoft</t>
+          <t xml:space="preserve">Named Credential hacia MuleSoft</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Setup &gt; Named Credentials &gt; endpoint del Mule (/api/v1/prices-and-inventory)</t>
+          <t xml:space="preserve">Setup &gt; Named Credentials &gt; endpoint del Mule (precios e inventario)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -572,7 +575,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metodo @AuraEnabled(continuation=true cacheable=true) devuelve new Continuation(120); con.addHttpRequest(callout:NC); callback tambien cacheable=true</t>
+          <t xml:space="preserve">El método @AuraEnabled(continuation=true cacheable=true) devuelve new Continuation(120); con.addHttpRequest(callout:NC); el callback también es cacheable</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -589,17 +592,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test del Continuation</t>
+          <t xml:space="preserve">Pruebas del Continuation</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test.setContinuationResponse(...) para cubrir sin SAP real</t>
+          <t xml:space="preserve">Test.setContinuationResponse(...) permite cubrir sin SAP real</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Testing Continuations</t>
+          <t xml:space="preserve">Testing de Continuations</t>
         </is>
       </c>
     </row>
@@ -616,7 +619,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Invoca Expression Set / Decision Matrix; retorna precio + impuesto de referencia</t>
+          <t xml:space="preserve">Invoca el Expression Set / Decision Matrix y retorna el precio e impuesto de referencia</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -638,12 +641,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crea Quote/QuoteLineItem u Order/OrderItem segun Record Type; bulkificado</t>
+          <t xml:space="preserve">Crea Quote/QuoteLineItem u Order/OrderItem según el Record Type; bulkificado</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quote &amp; Order Capture / Standalone Orders</t>
+          <t xml:space="preserve">Quote and Order Capture / Standalone Orders</t>
         </is>
       </c>
     </row>
@@ -655,12 +658,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SapOrderService (asincrono)</t>
+          <t xml:space="preserve">SapOrderService (asíncrono)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Queueable hace el callout de envio; al confirmar publica Sap_Order_Response__e</t>
+          <t xml:space="preserve">El Queueable realiza el callout de envío; al confirmar publica Sap_Order_Response__e</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -677,17 +680,17 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow de assetizacion</t>
+          <t xml:space="preserve">MaterialSearchService</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record-triggered al activar el Order: Asset + Vehicle(CurrentOwnerId) + Asset Contact Participant</t>
+          <t xml:space="preserve">Cascada de búsqueda: local &gt; SAP &gt; upsert &gt; extensión automática &gt; derivación a solicitud</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset lifecycle nativo</t>
+          <t xml:space="preserve">Ver columna 'Si NO encuentra' en Flujos</t>
         </is>
       </c>
     </row>
@@ -699,17 +702,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LWC pai ventaGuiadaAction</t>
+          <t xml:space="preserve">Flow de assetización</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">lightning__RecordAction + ScreenAction; recordId por setter; router por Record Type; empApi.subscribe</t>
+          <t xml:space="preserve">Record-triggered al activar el pedido: Asset + Vehicle (CurrentOwnerId) + Asset Contact Participant</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Screen Quick Action</t>
+          <t xml:space="preserve">Ciclo de vida nativo del Asset</t>
         </is>
       </c>
     </row>
@@ -721,17 +724,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LWC hijos por flujo</t>
+          <t xml:space="preserve">LWC padre ventaGuiadaAction</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finos; reusan servicios; invocacion IMPERATIVA del Continuation (para controlar cuando dispara)</t>
+          <t xml:space="preserve">lightning__RecordAction (ScreenAction); recordId por setter; router por Record Type; suscripción con empApi</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Call Apex Imperatively</t>
+          <t xml:space="preserve">Screen Quick Action</t>
         </is>
       </c>
     </row>
@@ -743,17 +746,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publicar la action en la Oportunidad</t>
+          <t xml:space="preserve">LWC hijos por línea de negocio</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Object Manager &gt; Opportunity &gt; New Action (Lightning Web Component) &gt; Lightning Record Page</t>
+          <t xml:space="preserve">Delgados; reutilizan los servicios; invocación imperativa del Continuation para controlar el disparo</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Call Apex Imperatively</t>
         </is>
       </c>
     </row>
@@ -765,42 +768,64 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Endurecer rendimiento</t>
+          <t xml:space="preserve">Publicar la acción</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">cacheable+LDS, Queueable, empApi, bulkify, Platform Cache, spinner/debounce</t>
+          <t xml:space="preserve">Object Manager &gt; Opportunity &gt; New Action (Lightning Web Component) &gt; Lightning Record Page</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ver hoja 'Estandares'</t>
+          <t xml:space="preserve">Quick Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Endurecer el rendimiento</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cacheable + LDS, Queueable, empApi, bulkificación, Platform Cache, spinner y debounce</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ver hoja Estándares</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF70AD47"/>
+  </sheetPr>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
     <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cobertura de flujos (mismos servicios, hijos distintos)</t>
+          <t xml:space="preserve">Flujos por línea de negocio — todos convergen en la creación de la cotización</t>
         </is>
       </c>
     </row>
@@ -810,7 +835,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flujo</t>
+          <t xml:space="preserve">Flujo / línea de negocio</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -825,135 +850,135 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP: sync / async</t>
+          <t xml:space="preserve">SAP: síncrono / asíncrono</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assetizacion</t>
+          <t xml:space="preserve">Assetización</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Si NO encuentra (busqueda sin resultado)</t>
+          <t xml:space="preserve">Si NO encuentra (búsqueda sin resultado)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Venta Vehiculo (Autos/Motos/Flotas)</t>
+          <t xml:space="preserve">Venta de Vehículo Nuevo (Autos / Motos / Flotas)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad &gt; action LWC</t>
+          <t xml:space="preserve">Oportunidad &gt; acción LWC</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle Inventory Search &gt; stock/precio SAP &gt; precio BRE &gt; Quote (RT Vehiculo) &gt; Order &gt; SAP</t>
+          <t xml:space="preserve">Vehicle Inventory Search &gt; stock y precio en SAP &gt; precio de referencia (BRE) &gt; Cotización (RT Vehículo) &gt; Pedido &gt; SAP</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sync: consulta (Continuation). Async: envio del pedido</t>
+          <t xml:space="preserve">Síncrono: consulta (Continuation). Asíncrono: envío del pedido</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset + Vehicle + Asset Contact Participant (360)</t>
+          <t xml:space="preserve">Asset + Vehicle + Asset Contact Participant (visión 360 del cliente)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unidad no disponible en la sucursal: Vehicle Inventory Search en OTRAS ubicaciones + Vehicle Transfer (nativos, licenciados). Accesorios/PA dentro de la venta siguen el arbol de material</t>
+          <t xml:space="preserve">Unidad no disponible en la sucursal: Vehicle Inventory Search en otras ubicaciones + Vehicle Transfer (nativos y licenciados). Los accesorios dentro de la venta siguen el árbol de material</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contraventa Repuestos</t>
+          <t xml:space="preserve">Venta de Usados</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record Type balcon (sin Oportunidad)</t>
+          <t xml:space="preserve">Oportunidad (línea Usados) &gt; acción LWC</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buscar pieza compatible por modelo/marca &gt; precio/stock SAP real-time &gt; Standalone Order &gt; SAP</t>
+          <t xml:space="preserve">Unidad del inventario de usados (HU-045: propia o en consignación) &gt; precio de la unidad según su ficha (lo administra Grupo Q, no SAP) &gt; Cotización &gt; Pedido &gt; SAP factura</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sync: consulta. Async: envio</t>
+          <t xml:space="preserve">Síncrono: disponibilidad de la unidad. Asíncrono: envío del pedido</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solo unidades serializables/garantizables</t>
+          <t xml:space="preserve">Nuevo Asset para el comprador; ConditionType pasa a Antiguo; el Vehicle es siempre el mismo (un VIN, una unidad)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arbol de material: verifica SAP &gt; existe para sociedad/centro: upsert Product2 (ProductCode) y sigue &gt; existe sin centro: extension automatica (HU-039) &gt; no existe: solicitud prellenada o vincular a la abierta (Follow). La venta sigue sin ese item</t>
+          <t xml:space="preserve">La unidad usada es única: búsqueda en el inventario de usados de otras sucursales (Inventory Search). Si es consignación: incorporación al inventario con aprobación del gerente, comisión según el contrato (Contract RT Consignación) y baja del inventario de consignación al cerrar la venta</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PA (Producto Automotriz / accesorios)</t>
+          <t xml:space="preserve">Contraventa de Repuestos (venta inmediata)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Igual a repuestos</t>
+          <t xml:space="preserve">Record Type de mostrador (sin Oportunidad)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compatibilidad por modelo/marca &gt; precio: SAP resuelve la lista aplicable (general/canal/cliente/volumen, con vigencia) &gt; Order &gt; SAP</t>
+          <t xml:space="preserve">Búsqueda de la pieza compatible por modelo y marca &gt; precio y stock en SAP en tiempo real &gt; Standalone Order &gt; SAP</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Listas de PA administradas en SAP (HU-028); PBE solo referencia de exhibicion. Precedencia de listas: pendiente confirmar con Grupo Q</t>
+          <t xml:space="preserve">Síncrono: consulta. Asíncrono: envío</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Si es serializable</t>
+          <t xml:space="preserve">Solo unidades serializables o con garantía</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mismo arbol de material que repuestos</t>
+          <t xml:space="preserve">Árbol de material: verificación en SAP &gt; si existe para la sociedad/centro se actualiza el catálogo y sigue &gt; si existe sin el centro, extensión automática (HU-039) &gt; si no existe, solicitud prellenada o vinculación a la abierta (Follow). La venta continúa sin ese ítem</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Venta Gestionada B2B (Repuestos &amp; PA)</t>
+          <t xml:space="preserve">Venta Gestionada B2B (Repuestos y PA)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opportunity pipeline GQOpportunityProcessRepuestosPA (mayoreo/flotas/cuentas clave/gobierno)</t>
+          <t xml:space="preserve">Pipeline de Oportunidad GQOpportunityProcessRepuestosPA (mayoreo, flotas, cuentas clave, gobierno)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visita en campo &gt; cotizacion con vigencia &gt; negociacion &gt; Order &gt; SAP</t>
+          <t xml:space="preserve">Visita en campo &gt; cotización con vigencia &gt; negociación &gt; Pedido &gt; SAP</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sync: consulta. Async: envio</t>
+          <t xml:space="preserve">Síncrono: consulta. Asíncrono: envío</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -963,93 +988,125 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mismo arbol de material; ventaja: la solicitud se sigue (Follow) y el item se cotiza despues dentro de la vigencia de la cotizacion</t>
+          <t xml:space="preserve">El mismo árbol de material; con la ventaja de que la solicitud se sigue (Follow) y el ítem se cotiza después, dentro de la vigencia de la cotización</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Combos (SKU con precio propio)</t>
+          <t xml:space="preserve">PA (Producto Automotriz / accesorios)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dentro de Repuestos/PA</t>
+          <t xml:space="preserve">Igual que repuestos</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El combo es un Product2 propio (ProductCode=material SAP); SAP resuelve su precio como cualquier material; disponibilidad del kit en HU-043</t>
+          <t xml:space="preserve">Compatibilidad por modelo y marca &gt; precio: SAP resuelve la lista aplicable (general, canal, cliente, volumen, con vigencia) &gt; Pedido &gt; SAP</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO requiere CPQ; la composicion no afecta el precio</t>
+          <t xml:space="preserve">Las listas de PA se administran en SAP (HU-028); el PricebookEntry es solo referencia de exhibición</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Si aplica</t>
+          <t xml:space="preserve">Si es serializable</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Combo no encontrado = mismo arbol de material (el combo es un material SAP)</t>
+          <t xml:space="preserve">El mismo árbol de material que repuestos</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuevo flujo (escalable)</t>
+          <t xml:space="preserve">Combos (SKU con precio propio)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Dentro de Repuestos y PA</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El combo es un Product2 propio (ProductCode = material SAP); SAP resuelve su precio como el de cualquier material; la disponibilidad del kit se resuelve en la HU-043</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No requiere CPQ; la composición no afecta el precio</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Si aplica</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combo no encontrado = el mismo árbol de material (el combo es un material SAP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flujo nuevo (escalable)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Nuevo hijo LWC</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reusa la capa de servicio Apex; solo cambia la UI</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reutiliza la capa de servicios Apex; solo cambia la interfaz</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Igual</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Igual</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reusa MaterialSearchService: el comportamiento sin-resultado es unico para todos los flujos</t>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reutiliza MaterialSearchService: el comportamiento de 'sin resultado' es único para todos los flujos</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFBF8F00"/>
+  </sheetPr>
   <cols>
-    <col min="1" max="1" width="46" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="1" max="1" width="48" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
     <col min="3" max="3" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision Sincrono vs Asincrono</t>
+          <t xml:space="preserve">Decisión: síncrono o asíncrono</t>
         </is>
       </c>
     </row>
@@ -1069,48 +1126,48 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por que</t>
+          <t xml:space="preserve">Por qué</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consulta precio+stock al SAP (el usuario espera la respuesta)</t>
+          <t xml:space="preserve">Consulta de precio y stock al SAP (el usuario espera la respuesta)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apex Continuation (invocacion imperativa)</t>
+          <t xml:space="preserve">Apex Continuation con invocación imperativa</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No bloquea la thread; 120s (vs 10s sincrono comun); hasta 3 callouts en paralelo</t>
+          <t xml:space="preserve">No bloquea el hilo; 120 segundos (contra 10 del síncrono común); hasta 3 callouts en paralelo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lectura de datos SF (Opp, Account, piezas compatibles)</t>
+          <t xml:space="preserve">Lectura de datos de Salesforce (Oportunidad, Cuenta, piezas compatibles)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">@wire + Lightning Data Service / Apex cacheable=true</t>
+          <t xml:space="preserve">@wire + Lightning Data Service / Apex cacheable</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cache, menos round-trips, sin Apex innecesario</t>
+          <t xml:space="preserve">Caché, menos viajes al servidor, sin Apex innecesario</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crear Quote / Order</t>
+          <t xml:space="preserve">Crear la cotización o el pedido</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1120,7 +1177,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accion puntual disparada por el usuario</t>
+          <t xml:space="preserve">Acción puntual disparada por el usuario</t>
         </is>
       </c>
     </row>
@@ -1132,19 +1189,19 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Queueable (asincrono)</t>
+          <t xml:space="preserve">Queueable (asíncrono)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El usuario no debe esperar la confirmacion del ERP</t>
+          <t xml:space="preserve">El usuario no debe esperar la confirmación del ERP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Devolver la confirmacion del SAP a la UI</t>
+          <t xml:space="preserve">Devolver la confirmación del SAP a la interfaz</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1154,14 +1211,14 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Push asincrono, sin polling</t>
+          <t xml:space="preserve">Push asíncrono, sin polling</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assetizacion tras la venta</t>
+          <t xml:space="preserve">Assetización tras la venta</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1171,27 +1228,44 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Declarativo, al activar el Order</t>
+          <t xml:space="preserve">Declarativo, al activarse el pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alerta de vencimiento del contrato de consignación</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flow con scheduled path sobre Contract.EndDate</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declarativo; el umbral lo define Grupo Q (HU-045)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFC00000"/>
+  </sheetPr>
   <cols>
-    <col min="1" max="1" width="130" customWidth="1"/>
+    <col min="1" max="1" width="135" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estandares y rendimiento (garantia de 'sin problemas ni lentitud')</t>
+          <t xml:space="preserve">Estándares y rendimiento</t>
         </is>
       </c>
     </row>
@@ -1201,91 +1275,91 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checklist obligatorio</t>
+          <t xml:space="preserve">Lista de verificación obligatoria</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Continuation para TODO callout externo. Nunca bloquear la thread del app server.</t>
+          <t xml:space="preserve">Continuation para todo callout externo; nunca bloquear el hilo del servidor.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">@AuraEnabled(continuation=true cacheable=true)  &lt;- espacio, NO coma. cacheable en toda la cadena, incluido el callback.</t>
+          <t xml:space="preserve">@AuraEnabled(continuation=true cacheable=true)  —  con espacio, no coma; cacheable en toda la cadena, incluido el callback.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">@wire + Lightning Data Service o cacheable=true para lecturas (cache).</t>
+          <t xml:space="preserve">@wire + Lightning Data Service o cacheable=true para las lecturas.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Queueable/asincrono para todo lo que el usuario no necesita esperar (envio al SAP, assetizacion).</t>
+          <t xml:space="preserve">Queueable / asíncrono para todo lo que el usuario no necesita esperar (envío al SAP, assetización).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platform Event + lightning/empApi para el resultado asincrono (sin polling).</t>
+          <t xml:space="preserve">Platform Event + lightning/empApi para el resultado asíncrono, sin polling.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bulkificar. Sin SOQL ni DML dentro de loops.</t>
+          <t xml:space="preserve">Bulkificación; sin SOQL ni DML dentro de bucles.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platform Cache / Custom Metadata para datos de referencia.</t>
+          <t xml:space="preserve">Platform Cache / Custom Metadata para los datos de referencia.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Named Credentials (seguridad + rendimiento). Nada de credenciales en codigo.</t>
+          <t xml:space="preserve">Named Credentials para la seguridad y el rendimiento; sin credenciales en el código.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spinner/skeleton, UI optimista, debounce en los inputs.</t>
+          <t xml:space="preserve">Spinner o skeleton, interfaz optimista y debounce en los campos de búsqueda.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reglas de negocio en BRE, no en Apex: mantenible por el negocio sin deploy.</t>
+          <t xml:space="preserve">Las reglas de negocio en el BRE, no en Apex: el negocio las mantiene sin despliegues.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test.setContinuationResponse(...) para cobertura de test sin SAP real.</t>
+          <t xml:space="preserve">Test.setContinuationResponse(...) para la cobertura de pruebas sin SAP real.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gobernanza: Apex/LWC solo en UI e integracion; nativo para modelo/cotizacion/pedido/assetizacion.</t>
+          <t xml:space="preserve">Gobernanza: LWC y Apex solo en interfaz e integración; lo nativo cubre el modelo, la cotización, el pedido y la assetización.</t>
         </is>
       </c>
     </row>
@@ -1295,49 +1369,49 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guardas de licenciamiento y fronteras (no olvidar)</t>
+          <t xml:space="preserve">Resguardos de licenciamiento y fronteras</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GrupoQ NO tiene CPQ, Revenue Cloud ni EPC. Ninguna HU debe asumirlos (HU-028 corregida: precio de combos y listas se resuelven en SAP + objetos estandar).</t>
+          <t xml:space="preserve">Grupo Q no tiene CPQ, Revenue Cloud ni EPC. Salesforce Pricing (app Price Management) tiene 1+1 asientos token: no se construye sobre él. El motor de reglas es el BRE (27.131 asientos de Designer y de Runtime, confirmados en la lista de licencias de la org).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra (no calcula ni convierte moneda). Listas de PA administradas en SAP; PBE solo referencia.</t>
+          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra; no calcula ni convierte moneda. Las listas de PA se administran en SAP; el PricebookEntry es referencia de exhibición.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carga masiva de precios/parametros de pricing: es del SAP (los datos viven alla). No construir herramienta de carga en Salesforce.</t>
+          <t xml:space="preserve">Usados: el precio de la unidad lo administra Grupo Q en la ficha del usado (HU-045); la factura sigue siendo de SAP. La consignación se modela con el Contract estándar (Record Type Consignación) — sin objetos custom.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Simulador de precios (FOB/factor/mark-up): variables viven en SAP; si Grupo Q quiere UI en Salesforce, exige servicio de simulacion expuesto por MuleSoft (agregar al contrato de integracion).</t>
+          <t xml:space="preserve">La carga masiva de precios y parámetros de pricing es del SAP; no se construye herramienta de carga en Salesforce.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparacion de precios multi-canal/sociedad: el endpoint del Mule debe aceptar consulta multi-contexto (agregar al contrato de integracion).</t>
+          <t xml:space="preserve">El simulador de precios (FOB, factor, mark-up) y la comparación multi-canal/sociedad exigen servicios expuestos por MuleSoft; van al contrato de integración.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">FUERA del flujo de ventas — dominio Gestion de Productos (HU-039): la creacion/extension de material NO es parte de este flujo. Unico punto de contacto: si la busqueda no encuentra el material, la UI ofrece registrar la solicitud y la venta continua. El servicio de escritura de dato maestro va al contrato MuleSoft del dominio de productos, no al de ventas.</t>
+          <t xml:space="preserve">Fuera del flujo de ventas — dominio de Gestión de Productos (HU-039): la creación y extensión de material no es parte de este flujo. Único punto de contacto: si la búsqueda no encuentra el material, la interfaz ofrece registrar la solicitud y la venta continúa.</t>
         </is>
       </c>
     </row>
@@ -1347,35 +1421,35 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limite a tener presente</t>
+          <t xml:space="preserve">Límite a tener presente</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Continuation con Named Credential funciona con auth de sistema (client credentials / API key). Si el Mule exige OAuth por-usuario, ajustar la estrategia de auth antes.</t>
+          <t xml:space="preserve">Continuation con Named Credential funciona con autenticación de sistema (client credentials o API key). Si el Mule exigiera OAuth por usuario, hay que ajustar la estrategia de autenticación antes de construir.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:A1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF7F7F7F"/>
+  </sheetPr>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="95" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referencias oficiales (fundamento de la solucion)</t>
+          <t xml:space="preserve">Referencias oficiales</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1483,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Continuations Example (LWC)</t>
+          <t xml:space="preserve">Ejemplo de Continuations (LWC)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1421,7 +1495,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">@AuraEnabled continuation</t>
+          <t xml:space="preserve">@AuraEnabled con continuation</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1433,7 +1507,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Long-Running Callouts (Apex Guide)</t>
+          <t xml:space="preserve">Callouts de larga duración (Apex)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1445,7 +1519,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Call Apex Imperatively (LWC)</t>
+          <t xml:space="preserve">Llamadas imperativas a Apex (LWC)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1469,7 +1543,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">lightning__RecordAction target</t>
+          <t xml:space="preserve">Target lightning__RecordAction</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1481,7 +1555,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automotive Cloud Standard Objects</t>
+          <t xml:space="preserve">Objetos estándar de Automotive Cloud</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1493,7 +1567,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create an Order from a Quote (QOCal)</t>
+          <t xml:space="preserve">Crear un pedido desde una cotización (QOCal)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1505,7 +1579,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">How Assets and Vehicles Are Related</t>
+          <t xml:space="preserve">Relación entre Assets y Vehicles</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1517,7 +1591,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create Asset Contact Participants</t>
+          <t xml:space="preserve">Asset Contact Participants</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1529,7 +1603,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create Products for Parts and Accessories</t>
+          <t xml:space="preserve">Productos para partes y accesorios</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1538,9 +1612,18 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criteria-Based Search and Filter</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/atlas.en-us.industries_reference.meta/industries_reference/criteria_based_search_and_filter_overview.htm</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Guia de ventas: ciclo del pedido (SAP no factura de inmediato) y cancelacion
Nueva hoja Ciclo del pedido: estados Borrador -> Enviado a SAP -> Confirmado
SAP -> Facturado -> Cancelado; la assetizacion se dispara unicamente al
llegar Facturado (correccion: antes estaba atada a la activacion). Nuevo
componente de retorno de facturacion inbound (MuleSoft actualiza el pedido).
Reglas de cancelacion por momento: antes de enviar (Salesforce), enviado sin
facturar (SAP anula via MuleSoft y se libera la unidad), ya facturado
(devolucion con nota de credito en SAP + Reduction Order estandar). Preguntas
para Grupo Q sobre aprobacion, ventana y devoluciones. Memoria actualizada.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -7,8 +7,9 @@
     <sheet name="Paso a paso" sheetId="3" r:id="rId3"/>
     <sheet name="Flujos" sheetId="4" r:id="rId4"/>
     <sheet name="Síncrono vs Asíncrono" sheetId="5" r:id="rId5"/>
-    <sheet name="Estándares" sheetId="6" r:id="rId6"/>
-    <sheet name="Referencias" sheetId="7" r:id="rId7"/>
+    <sheet name="Ciclo del pedido" sheetId="6" r:id="rId6"/>
+    <sheet name="Estándares" sheetId="7" r:id="rId7"/>
+    <sheet name="Referencias" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -429,64 +430,86 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow de assetización</t>
+          <t xml:space="preserve">Retorno de facturación (inbound)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow record-triggered</t>
+          <t xml:space="preserve">MuleSoft -&gt; Salesforce</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset + Vehicle (CurrentOwnerId) + Asset Contact Participant</t>
+          <t xml:space="preserve">Cuando SAP factura, MuleSoft actualiza el pedido: número de pedido SAP, número de factura y estado Facturado</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Declarativo, al activarse el pedido; sin objetos custom</t>
+          <t xml:space="preserve">API REST de Salesforce o Platform Event entrante; SAP no factura de inmediato — el pedido espera en Confirmado</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ventaGuiadaAction</t>
+          <t xml:space="preserve">Flow de assetización</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LWC padre</t>
+          <t xml:space="preserve">Flow record-triggered</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acción de pantalla; enruta por Record Type y contexto</t>
+          <t xml:space="preserve">Asset + Vehicle (CurrentOwnerId) + Asset Contact Participant</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">recordId por setter @api (no llega en connectedCallback)</t>
+          <t xml:space="preserve">Se dispara cuando el pedido pasa a FACTURADO (no al activarse); sin objetos custom</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">ventaGuiadaAction</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LWC padre</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Acción de pantalla; enruta por Record Type y contexto</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">recordId por setter @api (no llega en connectedCallback)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">ventaVehiculo / ventaUsados / contraventaRepuestos / ventaPA</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">LWC hijos</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Interfaz específica de cada línea de negocio</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Delgados; reutilizan la capa de servicios Apex</t>
         </is>
@@ -882,12 +905,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Síncrono: consulta (Continuation). Asíncrono: envío del pedido</t>
+          <t xml:space="preserve">Síncrono: consulta (Continuation). Asíncrono: envío del pedido y retorno de facturación</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset + Vehicle + Asset Contact Participant (visión 360 del cliente)</t>
+          <t xml:space="preserve">Tras la factura confirmada por SAP: Asset + Vehicle + Asset Contact Participant (visión 360 del cliente)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -914,12 +937,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Síncrono: disponibilidad de la unidad. Asíncrono: envío del pedido</t>
+          <t xml:space="preserve">Síncrono: disponibilidad de la unidad. Asíncrono: envío del pedido y retorno de facturación</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuevo Asset para el comprador; ConditionType pasa a Antiguo; el Vehicle es siempre el mismo (un VIN, una unidad)</t>
+          <t xml:space="preserve">Tras la factura confirmada por SAP: nuevo Asset para el comprador; ConditionType pasa a Antiguo; el Vehicle es siempre el mismo (un VIN, una unidad)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1218,32 +1241,66 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assetización tras la venta</t>
+          <t xml:space="preserve">Actualización del pedido cuando SAP factura</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow record-triggered</t>
+          <t xml:space="preserve">Inbound: MuleSoft actualiza el pedido (API REST o Platform Event)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Declarativo, al activarse el pedido</t>
+          <t xml:space="preserve">SAP no factura de inmediato; el evento de facturación llega después y dispara la assetización</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Assetización tras la venta</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flow record-triggered al pasar el pedido a Facturado</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declarativo; nunca antes de la factura confirmada</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cancelación de un pedido enviado a SAP</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitud vía MuleSoft; SAP anula y confirma</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP es el dueño del documento; Salesforce refleja el estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Alerta de vencimiento del contrato de consignación</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Flow con scheduled path sobre Contract.EndDate</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Declarativo; el umbral lo define Grupo Q (HU-045)</t>
         </is>
@@ -1254,6 +1311,279 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF7030A0"/>
+  </sheetPr>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="66" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ciclo de vida del pedido — SAP no factura de inmediato</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El pedido pasa por estados intermedios entre el envío y la factura. La assetización ocurre únicamente al llegar el estado Facturado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estado del pedido</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qué significa</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quién lo pone</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qué dispara</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borrador</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La cotización ganada generó el pedido</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salesforce</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nada aún</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enviado a SAP</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El pedido viajó vía MuleSoft</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salesforce (Queueable)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espera de la confirmación</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmado SAP</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP registró el pedido y devolvió su número</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retorno de MuleSoft</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se guarda el número de pedido SAP; el pedido espera la factura</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facturado</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP emitió la factura (número de factura)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retorno de MuleSoft (evento de facturación)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispara la assetización y la notificación al vendedor</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cancelado</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La cancelación fue confirmada</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Según la vía (ver reglas)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libera la unidad (Deallocated) y ajusta la Oportunidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reglas de cancelación (si el cliente la solicita)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momento</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qué se hace</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Responsable</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Antes de enviar a SAP</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se cancela en Salesforce; se libera la reserva de la unidad y se ajusta la Oportunidad</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salesforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enviado, pero aún NO facturado</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitud de cancelación vía MuleSoft; SAP anula el pedido y confirma; el pedido pasa a Cancelado y la unidad se libera</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salesforce solicita; SAP ejecuta</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya facturado</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya no es cancelación: es una devolución con nota de crédito en SAP. En Salesforce se registra con un pedido de reducción (Reduction Order estándar) y el Asset se ajusta según el desenlace</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP (documento fiscal); Salesforce refleja</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preguntas para Grupo Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">¿Quién puede solicitar y quién aprueba una cancelación? ¿Hay ventana de tiempo límite?</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al cancelar, ¿la unidad vuelve automáticamente a disponible para la venta o requiere revisión?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La devolución posterior a la factura, ¿entra en el alcance actual o se trata como proceso aparte?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFC00000"/>
@@ -1436,7 +1766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF7F7F7F"/>

</xml_diff>

<commit_message>
Guia de ventas: gobernanza de limites de Platform Events (punto de Davi)
La asignacion diaria de entrega se consume por suscriptor y hay tope de
clientes concurrentes. Reglas agregadas a Estandares: suscripcion acotada a
la sesion de la accion, filtros de canal por usuario/registro, retorno
tardio de factura por actualizacion de registro + Custom Notification (sin
limites de PE) y monitoreo con PlatformEventUsageMetric.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -1640,123 +1640,130 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platform Event + lightning/empApi para el resultado asíncrono, sin polling.</t>
+          <t xml:space="preserve">Platform Event + lightning/empApi para el resultado asíncrono, sin polling — con gobernanza de límites (punto de Davi): la asignación diaria de ENTREGA se consume por suscriptor (un evento entregado a N clientes cuenta N veces) y hay tope de clientes CometD concurrentes.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bulkificación; sin SOQL ni DML dentro de bucles.</t>
+          <t xml:space="preserve">Gobernanza de Platform Events: (1) suscripción acotada — la LWC se suscribe al enviar el pedido y se desuscribe al cerrar la acción, nunca todo el día; (2) filtros de canal (PlatformEventChannel con filtro por usuario/registro) para que cada suscriptor reciba SOLO sus eventos; (3) el retorno tardío (factura, horas o días después) NO usa empApi: llega por actualización del registro + Custom Notification (campana/push, sin límites de PE); (4) monitoreo con PlatformEventUsageMetric.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platform Cache / Custom Metadata para los datos de referencia.</t>
+          <t xml:space="preserve">Bulkificación; sin SOQL ni DML dentro de bucles.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Named Credentials para la seguridad y el rendimiento; sin credenciales en el código.</t>
+          <t xml:space="preserve">Platform Cache / Custom Metadata para los datos de referencia.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spinner o skeleton, interfaz optimista y debounce en los campos de búsqueda.</t>
+          <t xml:space="preserve">Named Credentials para la seguridad y el rendimiento; sin credenciales en el código.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Spinner o skeleton, interfaz optimista y debounce en los campos de búsqueda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Las reglas de negocio en el BRE, no en Apex: el negocio las mantiene sin despliegues.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Test.setContinuationResponse(...) para la cobertura de pruebas sin SAP real.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Gobernanza: LWC y Apex solo en interfaz e integración; lo nativo cubre el modelo, la cotización, el pedido y la assetización.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16"/>
-    </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Resguardos de licenciamiento y fronteras</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grupo Q no tiene CPQ, Revenue Cloud ni EPC. Salesforce Pricing (app Price Management) tiene 1+1 asientos token: no se construye sobre él. El motor de reglas es el BRE (27.131 asientos de Designer y de Runtime, confirmados en la lista de licencias de la org).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra; no calcula ni convierte moneda. Las listas de PA se administran en SAP; el PricebookEntry es referencia de exhibición.</t>
+          <t xml:space="preserve">Grupo Q no tiene CPQ, Revenue Cloud ni EPC. Salesforce Pricing (app Price Management) tiene 1+1 asientos token: no se construye sobre él. El motor de reglas es el BRE (27.131 asientos de Designer y de Runtime, confirmados en la lista de licencias de la org).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usados: el precio de la unidad lo administra Grupo Q en la ficha del usado (HU-045); la factura sigue siendo de SAP. La consignación se modela con el Contract estándar (Record Type Consignación) — sin objetos custom.</t>
+          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra; no calcula ni convierte moneda. Las listas de PA se administran en SAP; el PricebookEntry es referencia de exhibición.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">La carga masiva de precios y parámetros de pricing es del SAP; no se construye herramienta de carga en Salesforce.</t>
+          <t xml:space="preserve">Usados: el precio de la unidad lo administra Grupo Q en la ficha del usado (HU-045); la factura sigue siendo de SAP. La consignación se modela con el Contract estándar (Record Type Consignación) — sin objetos custom.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El simulador de precios (FOB, factor, mark-up) y la comparación multi-canal/sociedad exigen servicios expuestos por MuleSoft; van al contrato de integración.</t>
+          <t xml:space="preserve">La carga masiva de precios y parámetros de pricing es del SAP; no se construye herramienta de carga en Salesforce.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">El simulador de precios (FOB, factor, mark-up) y la comparación multi-canal/sociedad exigen servicios expuestos por MuleSoft; van al contrato de integración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Fuera del flujo de ventas — dominio de Gestión de Productos (HU-039): la creación y extensión de material no es parte de este flujo. Único punto de contacto: si la búsqueda no encuentra el material, la interfaz ofrece registrar la solicitud y la venta continúa.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24"/>
-    </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Límite a tener presente</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuation con Named Credential funciona con autenticación de sistema (client credentials o API key). Si el Mule exigiera OAuth por usuario, hay que ajustar la estrategia de autenticación antes de construir.</t>
         </is>

</xml_diff>

<commit_message>
Guia: numeros reales de Platform Events de la org (Enterprise, 22/07)
Pico real de entrega 345/dia frente a 25.000/dia default (1,4%); 2.000
clientes concurrentes; CDC con asignacion separada.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -1654,116 +1654,123 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bulkificación; sin SOQL ni DML dentro de bucles.</t>
+          <t xml:space="preserve">Verificado en la org (22/07/2026, Enterprise Edition): pico real de entrega de platform events = 345/día frente a la asignación default de 25.000/día (1,4%); tope de 2.000 clientes concurrentes. Los change events (CDC) tienen asignación separada. Con suscripción acotada y filtros de canal, la holgura es amplia incluso con crecimiento de 10x.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platform Cache / Custom Metadata para los datos de referencia.</t>
+          <t xml:space="preserve">Bulkificación; sin SOQL ni DML dentro de bucles.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Named Credentials para la seguridad y el rendimiento; sin credenciales en el código.</t>
+          <t xml:space="preserve">Platform Cache / Custom Metadata para los datos de referencia.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spinner o skeleton, interfaz optimista y debounce en los campos de búsqueda.</t>
+          <t xml:space="preserve">Named Credentials para la seguridad y el rendimiento; sin credenciales en el código.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Spinner o skeleton, interfaz optimista y debounce en los campos de búsqueda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Las reglas de negocio en el BRE, no en Apex: el negocio las mantiene sin despliegues.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Test.setContinuationResponse(...) para la cobertura de pruebas sin SAP real.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Gobernanza: LWC y Apex solo en interfaz e integración; lo nativo cubre el modelo, la cotización, el pedido y la assetización.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17"/>
-    </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Resguardos de licenciamiento y fronteras</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grupo Q no tiene CPQ, Revenue Cloud ni EPC. Salesforce Pricing (app Price Management) tiene 1+1 asientos token: no se construye sobre él. El motor de reglas es el BRE (27.131 asientos de Designer y de Runtime, confirmados en la lista de licencias de la org).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra; no calcula ni convierte moneda. Las listas de PA se administran en SAP; el PricebookEntry es referencia de exhibición.</t>
+          <t xml:space="preserve">Grupo Q no tiene CPQ, Revenue Cloud ni EPC. Salesforce Pricing (app Price Management) tiene 1+1 asientos token: no se construye sobre él. El motor de reglas es el BRE (27.131 asientos de Designer y de Runtime, confirmados en la lista de licencias de la org).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usados: el precio de la unidad lo administra Grupo Q en la ficha del usado (HU-045); la factura sigue siendo de SAP. La consignación se modela con el Contract estándar (Record Type Consignación) — sin objetos custom.</t>
+          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra; no calcula ni convierte moneda. Las listas de PA se administran en SAP; el PricebookEntry es referencia de exhibición.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">La carga masiva de precios y parámetros de pricing es del SAP; no se construye herramienta de carga en Salesforce.</t>
+          <t xml:space="preserve">Usados: el precio de la unidad lo administra Grupo Q en la ficha del usado (HU-045); la factura sigue siendo de SAP. La consignación se modela con el Contract estándar (Record Type Consignación) — sin objetos custom.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El simulador de precios (FOB, factor, mark-up) y la comparación multi-canal/sociedad exigen servicios expuestos por MuleSoft; van al contrato de integración.</t>
+          <t xml:space="preserve">La carga masiva de precios y parámetros de pricing es del SAP; no se construye herramienta de carga en Salesforce.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">El simulador de precios (FOB, factor, mark-up) y la comparación multi-canal/sociedad exigen servicios expuestos por MuleSoft; van al contrato de integración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Fuera del flujo de ventas — dominio de Gestión de Productos (HU-039): la creación y extensión de material no es parte de este flujo. Único punto de contacto: si la búsqueda no encuentra el material, la interfaz ofrece registrar la solicitud y la venta continúa.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25"/>
-    </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Límite a tener presente</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuation con Named Credential funciona con autenticación de sistema (client credentials o API key). Si el Mule exigiera OAuth por usuario, hay que ajustar la estrategia de autenticación antes de construir.</t>
         </is>

</xml_diff>

<commit_message>
Guia: TestDataFactory y mocks de integracion en Estandares (aporte de Davi)
Patron oficial de utilidades de prueba: TestDataFactory @isTest con metodos
por objeto, @TestSetup, fabrica de HttpCalloutMock para el Mule y
Test.setContinuationResponse. Utils pequena y cohesiva.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -1703,74 +1703,88 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Datos de prueba (aporte de Davi): clase TestDataFactory anotada @isTest (patrón oficial de utilidades de prueba), con métodos por objeto — p. ej. createQuoteWithVin(), createUsedVehicle(), createOrderConfirmado() — reutilizada por todas las clases de test vía @TestSetup. No cuenta para la cobertura y evita duplicar armado de datos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mocks de integración: una fábrica de HttpCalloutMock para las respuestas del Mule (precio/stock, confirmación, factura) + Test.setContinuationResponse. Clase de utilidades (Utils) pequeña y cohesiva — constantes y formato; la lógica vive en los servicios, no en Utils.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Gobernanza: LWC y Apex solo en interfaz e integración; lo nativo cubre el modelo, la cotización, el pedido y la assetización.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Resguardos de licenciamiento y fronteras</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grupo Q no tiene CPQ, Revenue Cloud ni EPC. Salesforce Pricing (app Price Management) tiene 1+1 asientos token: no se construye sobre él. El motor de reglas es el BRE (27.131 asientos de Designer y de Runtime, confirmados en la lista de licencias de la org).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra; no calcula ni convierte moneda. Las listas de PA se administran en SAP; el PricebookEntry es referencia de exhibición.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usados: el precio de la unidad lo administra Grupo Q en la ficha del usado (HU-045); la factura sigue siendo de SAP. La consignación se modela con el Contract estándar (Record Type Consignación) — sin objetos custom.</t>
+          <t xml:space="preserve">Grupo Q no tiene CPQ, Revenue Cloud ni EPC. Salesforce Pricing (app Price Management) tiene 1+1 asientos token: no se construye sobre él. El motor de reglas es el BRE (27.131 asientos de Designer y de Runtime, confirmados en la lista de licencias de la org).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">La carga masiva de precios y parámetros de pricing es del SAP; no se construye herramienta de carga en Salesforce.</t>
+          <t xml:space="preserve">Repuestos y PA: SAP es la fuente de la verdad del precio. Salesforce consulta y muestra; no calcula ni convierte moneda. Las listas de PA se administran en SAP; el PricebookEntry es referencia de exhibición.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El simulador de precios (FOB, factor, mark-up) y la comparación multi-canal/sociedad exigen servicios expuestos por MuleSoft; van al contrato de integración.</t>
+          <t xml:space="preserve">Usados: el precio de la unidad lo administra Grupo Q en la ficha del usado (HU-045); la factura sigue siendo de SAP. La consignación se modela con el Contract estándar (Record Type Consignación) — sin objetos custom.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">La carga masiva de precios y parámetros de pricing es del SAP; no se construye herramienta de carga en Salesforce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El simulador de precios (FOB, factor, mark-up) y la comparación multi-canal/sociedad exigen servicios expuestos por MuleSoft; van al contrato de integración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Fuera del flujo de ventas — dominio de Gestión de Productos (HU-039): la creación y extensión de material no es parte de este flujo. Único punto de contacto: si la búsqueda no encuentra el material, la interfaz ofrece registrar la solicitud y la venta continúa.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Límite a tener presente</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuation con Named Credential funciona con autenticación de sistema (client credentials o API key). Si el Mule exigiera OAuth por usuario, hay que ajustar la estrategia de autenticación antes de construir.</t>
         </is>

</xml_diff>

<commit_message>
Guia: proceso de admision de HUs nuevas y mapa vivo de historias
Dos hojas nuevas: 'Como encajar una HU' (los siete pasos repetibles:
resguardos, flujo, modelo, fronteras, tareas, registro, parecer) y 'Mapa de
HUs' (indice de 14 historias con donde encaja cada una, estado y nota).
Objetivo: ninguna historia nueva se analiza desde cero ni contradice lo
decidido — el trabajo pasa a ser clasificacion.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -9,7 +9,9 @@
     <sheet name="Síncrono vs Asíncrono" sheetId="5" r:id="rId5"/>
     <sheet name="Ciclo del pedido" sheetId="6" r:id="rId6"/>
     <sheet name="Estándares" sheetId="7" r:id="rId7"/>
-    <sheet name="Referencias" sheetId="8" r:id="rId8"/>
+    <sheet name="Cómo encajar una HU" sheetId="8" r:id="rId8"/>
+    <sheet name="Mapa de HUs" sheetId="9" r:id="rId9"/>
+    <sheet name="Referencias" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -229,6 +231,198 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF7F7F7F"/>
+  </sheetPr>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="95" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencias oficiales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tema</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">URL oficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Continuations (LWC)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/apex-continuations.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ejemplo de Continuations (LWC)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/apex-continuations-component-example.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@AuraEnabled con continuation</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/apex-continuations-auraenabled.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Callouts de larga duración (Apex)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/atlas.en-us.apexcode.meta/apexcode/apex_continuation_overview.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Llamadas imperativas a Apex (LWC)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/apex-call-imperative.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Screen Quick Actions (LWC)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/use-quick-actions-screen.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Target lightning__RecordAction</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/targets-lightning-record-action.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objetos estándar de Automotive Cloud</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/atlas.en-us.automotive_cloud.meta/automotive_cloud/automotive_objects.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crear un pedido desde una cotización (QOCal)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=ind.qocal_create_orders_from_a_quote.htm&amp;language=en_US&amp;type=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Relación entre Assets y Vehicles</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=sf.auto_relationship_assets_vehicles.htm&amp;language=en_US&amp;type=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asset Contact Participants</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=sf.auto_create_asset_contact_participants.htm&amp;language=en_US&amp;type=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Productos para partes y accesorios</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=sf.auto_products_parts_accessories.htm&amp;language=en_US&amp;type=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criteria-Based Search and Filter</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://developer.salesforce.com/docs/atlas.en-us.industries_reference.meta/industries_reference/criteria_based_search_and_filter_overview.htm</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1797,188 +1991,644 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF7F7F7F"/>
+    <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="95" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referencias oficiales</t>
+          <t xml:space="preserve">Cómo encajar una HU nueva (proceso de admisión — repetible)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cada historia nueva pasa por estos siete pasos, en orden. El objetivo: ninguna HU se analiza desde cero ni contradice lo ya decidido; el trabajo es clasificar, no reinventar.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tema</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">URL oficial</t>
-        </is>
-      </c>
+      <c r="A3"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Continuations (LWC)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/apex-continuations.html</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paso</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qué se hace</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contra qué se valida</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salida</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ejemplo de Continuations (LWC)</t>
+          <t xml:space="preserve">1. Resguardos</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/apex-continuations-component-example.html</t>
+          <t xml:space="preserve">Verificar que la HU no asuma CPQ, Revenue Cloud, EPC ni el app Price Management (1+1 asientos token). Motor de reglas = BRE; sin objetos custom nuevos; sin Case en Repuestos.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hoja Estándares — Resguardos de licenciamiento</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU corregida o aprobada en licenciamiento</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">@AuraEnabled con continuation</t>
+          <t xml:space="preserve">2. Flujo</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/apex-continuations-auraenabled.html</t>
+          <t xml:space="preserve">Identificar a cuál de los flujos de la hoja Flujos pertenece (Vehículo Nuevo, Usados, Contraventa, Gestionada B2B, PA, Combos) — o si toca otro dominio (productos, impuestos).</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hoja Flujos</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La HU queda anclada a un flujo (o marcada fuera del flujo de ventas)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Callouts de larga duración (Apex)</t>
+          <t xml:space="preserve">3. Modelo</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/atlas.en-us.apexcode.meta/apexcode/apex_continuation_overview.htm</t>
+          <t xml:space="preserve">Mapear cada concepto de la HU a lo nativo ANTES de crear campos: describe primero, campo después solo si no existe.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Describes de la org + Object Reference</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lista de objetos/campos: nativo reutilizado vs custom justificado</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Llamadas imperativas a Apex (LWC)</t>
+          <t xml:space="preserve">4. Fronteras</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/apex-call-imperative.html</t>
+          <t xml:space="preserve">Marcar qué NO es de la HU (reserva, proforma, descuentos, etc.) y las dependencias con otras HUs. Los GAP se declaran, no se asumen.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mapa de HUs</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sección de fronteras y dependencias explícita</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Screen Quick Actions (LWC)</t>
+          <t xml:space="preserve">5. Tareas</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/use-quick-actions-screen.html</t>
+          <t xml:space="preserve">Generar la planilla de tareas técnicas (formato estándar: ID, tipo, nativo/custom, dependencia, estimación) con la columna 'Puede iniciar ya' (verde) vs 'espera' (naranja).</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Formato HU036/HU042_Tarefas_Tecnicas</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planilla de tareas con lo liberado y lo bloqueado</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Target lightning__RecordAction</t>
+          <t xml:space="preserve">6. Registro</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/platform/lwc/guide/targets-lightning-record-action.html</t>
+          <t xml:space="preserve">Toda decisión nueva que la HU genere entra el MISMO día en esta guía y en la memoria del proyecto. Si contradice algo ya travado, se resuelve antes del refinamiento — nunca en la sesión con el cliente.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esta guía + CLAUDE.md del repo</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guía y memoria actualizadas; una sola versión de la verdad</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objetos estándar de Automotive Cloud</t>
+          <t xml:space="preserve">7. Parecer</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/atlas.en-us.automotive_cloud.meta/automotive_cloud/automotive_objects.htm</t>
+          <t xml:space="preserve">Emitir la validación para Melisa: qué está bien, qué se ajusta antes del Jira, qué pregunta queda para Grupo Q (con respuesta sugerida).</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Todo lo anterior</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU validada — versión única y alineada para el refinamiento</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFD9A400"/>
+  </sheetPr>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="56" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mapa de HUs — dónde encaja cada historia (índice vivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cada HU nueva entra en este mapa al pasar por el proceso de admisión. Si una historia no encaja en ningún flujo ni dominio, es señal de alcance nuevo: se discute antes de refinar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tema</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dónde encaja</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estado</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU-016</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oportunidad — lookup de Vehículo</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Venta Vehículo (base)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Construida</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opportunity.Vehiculo__c existente; reutilizado por la HU-042 para usados</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU-027</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Integración M365 / correo</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fuera del flujo de ventas</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En desbloqueo</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plan propio (Graph-first) con el admin de Grupo Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU-028</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precio de Repuestos y PA</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contraventa / PA / Gestionada B2B</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validada con ajustes</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP fuente de la verdad del precio; sin CPQ; listas de PA en SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU-030</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Catálogo de productos (maestro)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dominio de productos</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dependencia</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provee el maestro que consumen la búsqueda y la HU-039</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU-031</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificación y búsqueda de productos</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contraventa / PA (búsqueda)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comportamiento 'sin resultado' definido (árbol de material)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU-036</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avalúo del usado (trade-in)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Venta de Usados (entrada)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tareas técnicas listas</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Familia nativa Appraisal + Scheduler; alimenta el inventario de la HU-045</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU-038</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Listas de precios y campos comerciales</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transversal de precios</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En sesión con el cliente</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workbook de la sesión integral v4; la lógica del QRM migra a BRE + Pricebook</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crear un pedido desde una cotización (QOCal)</t>
+          <t xml:space="preserve">HU-039</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=ind.qocal_create_orders_from_a_quote.htm&amp;language=en_US&amp;type=5</t>
+          <t xml:space="preserve">Solicitud de creación de material</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dominio de productos (contacto: búsqueda)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validada</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product2 RT Solicitud; sin objeto custom; retorno graba el MATNR</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relación entre Assets y Vehicles</t>
+          <t xml:space="preserve">HU-042</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=sf.auto_relationship_assets_vehicles.htm&amp;language=en_US&amp;type=5</t>
+          <t xml:space="preserve">Selección de vehículo a cotizar</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Venta Vehículo Nuevo / Usados / Motos</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En construcción</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verde en curso (describe listo, matrices BRE); pantallas esperan validación</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset Contact Participants</t>
+          <t xml:space="preserve">HU-043</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=sf.auto_create_asset_contact_participants.htm&amp;language=en_US&amp;type=5</t>
+          <t xml:space="preserve">Disponibilidad y líneas al cotizar</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Venta (post-selección)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resuelve stock/reservas y disponibilidad de kits (combos)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Productos para partes y accesorios</t>
+          <t xml:space="preserve">HU-045</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=sf.auto_products_parts_accessories.htm&amp;language=en_US&amp;type=5</t>
+          <t xml:space="preserve">Registro de usados y consignación</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Venta de Usados (inventario)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validada con ajustes</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contract RT Consignación; misma unidad Vehicle por VIN; Asset por episodio</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Criteria-Based Search and Filter</t>
+          <t xml:space="preserve">HU-046</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://developer.salesforce.com/docs/atlas.en-us.industries_reference.meta/industries_reference/criteria_based_search_and_filter_overview.htm</t>
+          <t xml:space="preserve">Vehículo demo / exhibición y estados</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reserva (estados de inventario)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente de validar</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modelagem del demo lista (AllocationStatus + Vehicle.Status); bloqueos viven aquí, no en la cotización</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HU-059</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proforma y envío de la cotización</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Venta (emisión)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF vía Document Generation; envío por correo con versionado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contraventa</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nueva Contra-Venda (transaccional)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contraventa inmediata</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Funcional cerrado</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Construcción espera la validación de arquitectura; RT Contraventa Repuestos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Guia: HU-014 en el Mapa de HUs y resguardo de componentes con HU de origen
HU-014 (cliente ocasional/Golden Record) registrada esperando definicion de
Grupo Q; componentes de Order de la actividad de Wilmar marcados para
remodelar con la HU y retirados del paquete DLG. Resguardo nuevo: todo
componente creado se registra el mismo dia con su HU de origen; sin dueno
rastreable no entra en paquete de deploy.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -1968,17 +1968,24 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28"/>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Todo componente creado (campo, validación, flow) se registra el MISMO día en esta guía con su HU de origen y Description llena. Componente sin dueño rastreable no entra en ningún paquete de deploy — caso HU-014/Order (22/07): campos creados fuera del funil terminaron en el paquete de otra frente.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Límite a tener presente</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuation con Named Credential funciona con autenticación de sistema (client credentials o API key). Si el Mule exigiera OAuth por usuario, hay que ajustar la estrategia de autenticación antes de construir.</t>
         </is>
@@ -2257,376 +2264,403 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-016</t>
+          <t xml:space="preserve">HU-014</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad — lookup de Vehículo</t>
+          <t xml:space="preserve">Cuenta/contacto en mostrador y cliente ocasional</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Venta Vehículo (base)</t>
+          <t xml:space="preserve">Contraventa (alta de cliente)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Construida</t>
+          <t xml:space="preserve">Esperando definición de Grupo Q</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opportunity.Vehiculo__c existente; reutilizado por la HU-042 para usados</t>
+          <t xml:space="preserve">Datos mínimos y uso fiscal del ocasional pendientes; modelo ancla en Account/Contact (Golden Record). Componentes creados en Order (actividad Wilmar) se remodelan con esta HU — retirados del paquete DLG</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-027</t>
+          <t xml:space="preserve">HU-016</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integración M365 / correo</t>
+          <t xml:space="preserve">Oportunidad — lookup de Vehículo</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fuera del flujo de ventas</t>
+          <t xml:space="preserve">Venta Vehículo (base)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">En desbloqueo</t>
+          <t xml:space="preserve">Construida</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plan propio (Graph-first) con el admin de Grupo Q</t>
+          <t xml:space="preserve">Opportunity.Vehiculo__c existente; reutilizado por la HU-042 para usados</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-028</t>
+          <t xml:space="preserve">HU-027</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio de Repuestos y PA</t>
+          <t xml:space="preserve">Integración M365 / correo</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contraventa / PA / Gestionada B2B</t>
+          <t xml:space="preserve">Fuera del flujo de ventas</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validada con ajustes</t>
+          <t xml:space="preserve">En desbloqueo</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP fuente de la verdad del precio; sin CPQ; listas de PA en SAP</t>
+          <t xml:space="preserve">Plan propio (Graph-first) con el admin de Grupo Q</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-030</t>
+          <t xml:space="preserve">HU-028</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catálogo de productos (maestro)</t>
+          <t xml:space="preserve">Precio de Repuestos y PA</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dominio de productos</t>
+          <t xml:space="preserve">Contraventa / PA / Gestionada B2B</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dependencia</t>
+          <t xml:space="preserve">Validada con ajustes</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provee el maestro que consumen la búsqueda y la HU-039</t>
+          <t xml:space="preserve">SAP fuente de la verdad del precio; sin CPQ; listas de PA en SAP</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-031</t>
+          <t xml:space="preserve">HU-030</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificación y búsqueda de productos</t>
+          <t xml:space="preserve">Catálogo de productos (maestro)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contraventa / PA (búsqueda)</t>
+          <t xml:space="preserve">Dominio de productos</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Dependencia</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comportamiento 'sin resultado' definido (árbol de material)</t>
+          <t xml:space="preserve">Provee el maestro que consumen la búsqueda y la HU-039</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-036</t>
+          <t xml:space="preserve">HU-031</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avalúo del usado (trade-in)</t>
+          <t xml:space="preserve">Identificación y búsqueda de productos</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Venta de Usados (entrada)</t>
+          <t xml:space="preserve">Contraventa / PA (búsqueda)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tareas técnicas listas</t>
+          <t xml:space="preserve">En curso</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Familia nativa Appraisal + Scheduler; alimenta el inventario de la HU-045</t>
+          <t xml:space="preserve">Comportamiento 'sin resultado' definido (árbol de material)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-038</t>
+          <t xml:space="preserve">HU-036</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Listas de precios y campos comerciales</t>
+          <t xml:space="preserve">Avalúo del usado (trade-in)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transversal de precios</t>
+          <t xml:space="preserve">Venta de Usados (entrada)</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">En sesión con el cliente</t>
+          <t xml:space="preserve">Tareas técnicas listas</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Workbook de la sesión integral v4; la lógica del QRM migra a BRE + Pricebook</t>
+          <t xml:space="preserve">Familia nativa Appraisal + Scheduler; alimenta el inventario de la HU-045</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-039</t>
+          <t xml:space="preserve">HU-038</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solicitud de creación de material</t>
+          <t xml:space="preserve">Listas de precios y campos comerciales</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dominio de productos (contacto: búsqueda)</t>
+          <t xml:space="preserve">Transversal de precios</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validada</t>
+          <t xml:space="preserve">En sesión con el cliente</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2 RT Solicitud; sin objeto custom; retorno graba el MATNR</t>
+          <t xml:space="preserve">Workbook de la sesión integral v4; la lógica del QRM migra a BRE + Pricebook</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-042</t>
+          <t xml:space="preserve">HU-039</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selección de vehículo a cotizar</t>
+          <t xml:space="preserve">Solicitud de creación de material</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Venta Vehículo Nuevo / Usados / Motos</t>
+          <t xml:space="preserve">Dominio de productos (contacto: búsqueda)</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">En construcción</t>
+          <t xml:space="preserve">Validada</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verde en curso (describe listo, matrices BRE); pantallas esperan validación</t>
+          <t xml:space="preserve">Product2 RT Solicitud; sin objeto custom; retorno graba el MATNR</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-043</t>
+          <t xml:space="preserve">HU-042</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disponibilidad y líneas al cotizar</t>
+          <t xml:space="preserve">Selección de vehículo a cotizar</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Venta (post-selección)</t>
+          <t xml:space="preserve">Venta Vehículo Nuevo / Usados / Motos</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendiente</t>
+          <t xml:space="preserve">En construcción</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resuelve stock/reservas y disponibilidad de kits (combos)</t>
+          <t xml:space="preserve">Verde en curso (describe listo, matrices BRE); pantallas esperan validación</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-045</t>
+          <t xml:space="preserve">HU-043</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registro de usados y consignación</t>
+          <t xml:space="preserve">Disponibilidad y líneas al cotizar</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Venta de Usados (inventario)</t>
+          <t xml:space="preserve">Venta (post-selección)</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validada con ajustes</t>
+          <t xml:space="preserve">Pendiente</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contract RT Consignación; misma unidad Vehicle por VIN; Asset por episodio</t>
+          <t xml:space="preserve">Resuelve stock/reservas y disponibilidad de kits (combos)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-046</t>
+          <t xml:space="preserve">HU-045</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehículo demo / exhibición y estados</t>
+          <t xml:space="preserve">Registro de usados y consignación</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reserva (estados de inventario)</t>
+          <t xml:space="preserve">Venta de Usados (inventario)</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendiente de validar</t>
+          <t xml:space="preserve">Validada con ajustes</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelagem del demo lista (AllocationStatus + Vehicle.Status); bloqueos viven aquí, no en la cotización</t>
+          <t xml:space="preserve">Contract RT Consignación; misma unidad Vehicle por VIN; Asset por episodio</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-059</t>
+          <t xml:space="preserve">HU-046</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proforma y envío de la cotización</t>
+          <t xml:space="preserve">Vehículo demo / exhibición y estados</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Venta (emisión)</t>
+          <t xml:space="preserve">Reserva (estados de inventario)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendiente</t>
+          <t xml:space="preserve">Pendiente de validar</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PDF vía Document Generation; envío por correo con versionado</t>
+          <t xml:space="preserve">Modelagem del demo lista (AllocationStatus + Vehicle.Status); bloqueos viven aquí, no en la cotización</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">HU-059</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proforma y envío de la cotización</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Venta (emisión)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF vía Document Generation; envío por correo con versionado</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Contraventa</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Nueva Contra-Venda (transaccional)</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Contraventa inmediata</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Funcional cerrado</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Construcción espera la validación de arquitectura; RT Contraventa Repuestos</t>
         </is>

</xml_diff>

<commit_message>
Guia: confirmaciones del indice oficial de objetos estandar
AssetAccountParticipant/AssetContactParticipant oficiales (API name de la
HU-045 resuelto); ProductRelatedMaterial como ancla de compatibilidad
pieza-modelo; ReturnOrder/ReturnOrderLineItem agregados a la devolucion
pos-factura en el Ciclo del pedido.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -1733,7 +1733,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ya no es cancelación: es una devolución con nota de crédito en SAP. En Salesforce se registra con un pedido de reducción (Reduction Order estándar) y el Asset se ajusta según el desenlace</t>
+          <t xml:space="preserve">Ya no es cancelación: es una devolución con nota de crédito en SAP. En Salesforce: Reduction Order estándar (ajuste comercial) y, si la unidad retorna al inventario, ReturnOrder / ReturnOrderLineItem (retorno físico, API 60+); el Asset se ajusta según el desenlace</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1975,17 +1975,24 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29"/>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmado en el índice oficial de objetos (23/07): AssetAccountParticipant y AssetContactParticipant existen como junctions estándar (API 59+) — resuelve el API name pendiente de la HU-045 (consignante). ProductRelatedMaterial (API 55+) es el objeto oficial de componentes de un producto — ancla nativa de la compatibilidad pieza-modelo. ReturnOrder/ReturnOrderLineItem (API 60+) cubren el retorno físico al inventario.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Límite a tener presente</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuation con Named Credential funciona con autenticación de sistema (client credentials o API key). Si el Mule exigiera OAuth por usuario, hay que ajustar la estrategia de autenticación antes de construir.</t>
         </is>

</xml_diff>

<commit_message>
Guia: referencia de MuleSoft Direct para Automotive Cloud
Assets pre-construidos (Connected Vehicles, STAR, Service Process) anotados
en Referencias; los contratos SAP del proyecto siguen como APIs propias en
el Anypoint del cliente.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
+++ b/deploy/arquitetura-ventas/GUIA-LWC-APEX-VENTAS.xlsx
@@ -419,6 +419,18 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MuleSoft Direct para Automotive Cloud (assets: Connected Vehicles, STAR, Service Process)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://help.salesforce.com/s/articleView?id=sf.industry_integration_solutions.htm&amp;type=5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>